<commit_message>
fix: use standard column width defaults
Change baseColWidth from 30 to 7.58 and add explicit <cols> definition
setting all columns to width 7.58, matching Excel's standard default.
</commit_message>
<xml_diff>
--- a/test/test.xlsx
+++ b/test/test.xlsx
@@ -71,7 +71,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetFormatPr baseColWidth="30" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="7.58" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="16384" width="7.58" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="inlineStr">

</xml_diff>

<commit_message>
fix: use built-in date format instead of custom numFmt 170
Replace custom numFmtId 170 (yyyy-mm-dd hh:mm:ss) with built-in
numFmtId 14 (mm-dd-yy) at cellXfs index 6. Remove the custom numFmt
definition since it's no longer needed.
</commit_message>
<xml_diff>
--- a/test/test.xlsx
+++ b/test/test.xlsx
@@ -15,9 +15,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <numFmts count="1">
-    <numFmt numFmtId="170" formatCode="yyyy-mm-dd hh:mm:ss"/>
-  </numFmts>
+  <numFmts count="0">
+    </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -54,7 +53,7 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>

</xml_diff>